<commit_message>
Card Spread sheet updated
</commit_message>
<xml_diff>
--- a/Rules/Mage Knight Card and Skill texts .xlsx
+++ b/Rules/Mage Knight Card and Skill texts .xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/18c549927b9fc512/Board Games/Mage Knight/TTS/Lua Code/Mage_Knight_Highly_Scripted/Rules/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="394" documentId="13_ncr:1_{34FC8D39-88EA-4E94-97D8-6F4E26FD2FAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{244E99E0-54D9-4CC1-9F7F-322150D79929}"/>
+  <xr:revisionPtr revIDLastSave="645" documentId="13_ncr:1_{34FC8D39-88EA-4E94-97D8-6F4E26FD2FAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E95CCC8D-27BA-408E-AA4A-690B0DACBA43}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Starting Cards" sheetId="9" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1289" uniqueCount="1119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1480" uniqueCount="1208">
   <si>
     <t>Set</t>
   </si>
@@ -3216,9 +3216,6 @@
 During the block phase of combat, you may spend this unit to cancel one attack. If you do, fame +1. </t>
   </si>
   <si>
-    <t xml:space="preserve">Skip the block and damage assigning phases of this combat. </t>
-  </si>
-  <si>
     <t xml:space="preserve">Assign this to a unit you control.
 The assigned unit gets armor +1, fire resistance and ice resistance. </t>
   </si>
@@ -3265,14 +3262,6 @@
 Enemies lose physical resistance this turn. Fame +1 for each enemy you defeat this turn. </t>
   </si>
   <si>
-    <t xml:space="preserve">Siege Attack 6.
-Roll a mana die. If you roll black or red, you get a Wound. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Siege Attack 6.
-You may add up to +6 to this Siege Attack. For each +1 you added roll a mana die. You get a Wound for each black or red rolled. </t>
-  </si>
-  <si>
     <t xml:space="preserve">Heal 2.
 Fame +1 for each point of Healing provided by this card you spend this turn. </t>
   </si>
@@ -3325,14 +3314,6 @@
   </si>
   <si>
     <t xml:space="preserve">Gain Fame +2.  Recruit any one Unit from the Units offer for free.  (If you are at your Command limit, you must disband one of your units first.) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Assign this to a unit you control.
-Once a Round, when the Unit is about to get wounded, flip this card to ignore the Wound and any additional effects from it.  The Unit can still only be assigned damage once each combat. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anytime except during combat:
-Heal all of your Units completely. </t>
   </si>
   <si>
     <t xml:space="preserve">Attack 3.  For one enemy defeated by this attack gain one crystal to your inventory. It may be red if the enemy had Fire Resistance, blue if it had Ice Resistance, green if it had Physical Resistance.  You may always choose white. </t>
@@ -3369,12 +3350,6 @@
     <t xml:space="preserve">Discard a card of any color.  Use the stronger effect of a Spell of the same color from the Spells offer without paying its mana cost.  You may do so even during the Day. </t>
   </si>
   <si>
-    <t>Remove and reveal the top card of the Artifacts deck. This turn, you may use Mysterious Box as if it was that Artifact. If you do then Fame +1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">At the end of the turn: put the revealed Artifact on the bottom of the Artifacts deck; if you did not use Mysterious Box then put it back in your hand; if you placed it on an unit as a banner then discard it. </t>
-  </si>
-  <si>
     <t>Silver Units</t>
   </si>
   <si>
@@ -3972,6 +3947,315 @@
   </si>
   <si>
     <t>Target enemy does not attack this combat. You may target additional enemies: pay 1 move point for the second enemy, pay 2 move point for the third enemy, etc.</t>
+  </si>
+  <si>
+    <t>2eb8d1</t>
+  </si>
+  <si>
+    <t>2eb8d7</t>
+  </si>
+  <si>
+    <t>2eb8e0</t>
+  </si>
+  <si>
+    <t>2eb8e8</t>
+  </si>
+  <si>
+    <t>2eb8d2</t>
+  </si>
+  <si>
+    <t>2eb8f4</t>
+  </si>
+  <si>
+    <t>8907d7</t>
+  </si>
+  <si>
+    <t>2eb8f5</t>
+  </si>
+  <si>
+    <t>2eb8f3</t>
+  </si>
+  <si>
+    <t>2eb8e6</t>
+  </si>
+  <si>
+    <t>2eb8e1</t>
+  </si>
+  <si>
+    <t>47e71c</t>
+  </si>
+  <si>
+    <t>2eb8d9</t>
+  </si>
+  <si>
+    <t>7d608f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assign this to a unit you control. Once a Round, when the Unit is about to get wounded, flip this card to ignore the Wound and any additional effects from it.  The Unit can still only be assigned damage once each combat. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anytime except during combat:
+Heal all of your Units completely. </t>
+  </si>
+  <si>
+    <t>98681f</t>
+  </si>
+  <si>
+    <t>085e68</t>
+  </si>
+  <si>
+    <t>085e66</t>
+  </si>
+  <si>
+    <t>085e67</t>
+  </si>
+  <si>
+    <t>085e63</t>
+  </si>
+  <si>
+    <t>085e64</t>
+  </si>
+  <si>
+    <t>085e65</t>
+  </si>
+  <si>
+    <t>085e69</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove and reveal the top card of the Artifacts deck. This turn, you may use Mysterious Box as if it was that Artifact. If you do then Fame +1.
+At the end of the turn: put the revealed Artifact on the bottom of the Artifacts deck; if you did not use Mysterious Box then put it back in your hand; if you placed it on an unit as a banner then discard it. </t>
+  </si>
+  <si>
+    <t>085e59</t>
+  </si>
+  <si>
+    <t>085e56</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Siege Attack 5.
+Roll a mana die. If you roll black or red, you get a Wound. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Siege Attack 5.
+You may add up to +5 to this Siege Attack. For each +1 you added roll a mana die. You get a Wound for each black or red rolled. </t>
+  </si>
+  <si>
+    <t>085e55</t>
+  </si>
+  <si>
+    <t>085e57</t>
+  </si>
+  <si>
+    <t>085e61</t>
+  </si>
+  <si>
+    <t>085e62</t>
+  </si>
+  <si>
+    <t>085e58</t>
+  </si>
+  <si>
+    <t>085e60</t>
+  </si>
+  <si>
+    <t>085e50</t>
+  </si>
+  <si>
+    <t>df2eae</t>
+  </si>
+  <si>
+    <t>7b9ec1</t>
+  </si>
+  <si>
+    <t>Up to 3 enemies do not attack this combat.</t>
+  </si>
+  <si>
+    <t>6b4654</t>
+  </si>
+  <si>
+    <t>085e52</t>
+  </si>
+  <si>
+    <t>085e51</t>
+  </si>
+  <si>
+    <t>085e54</t>
+  </si>
+  <si>
+    <t>085e53</t>
+  </si>
+  <si>
+    <t>dea60c</t>
+  </si>
+  <si>
+    <t>Tranquility</t>
+  </si>
+  <si>
+    <t>Heal 1 or draw a card.</t>
+  </si>
+  <si>
+    <t>Heal 2 or draw two cards.</t>
+  </si>
+  <si>
+    <t>Concentration</t>
+  </si>
+  <si>
+    <t>Gain a blue, white or red mana token.</t>
+  </si>
+  <si>
+    <t>When you play this play another Action card with it. Get the stronger effect of that card for free. If that effect gives you move, Influence, Block, or any type of Attack, get that amount plus 2.</t>
+  </si>
+  <si>
+    <t>March</t>
+  </si>
+  <si>
+    <t>Move 4</t>
+  </si>
+  <si>
+    <t>Infamous Reprisals</t>
+  </si>
+  <si>
+    <t>Mevok</t>
+  </si>
+  <si>
+    <t>Mana Draw</t>
+  </si>
+  <si>
+    <t>You can use one additional mana die from the Source this turn.</t>
+  </si>
+  <si>
+    <t>Take a mana die from the Source and set it to any color except gold. Gain two mana tokens of that color. Do not reroll this die when you return it to the source.</t>
+  </si>
+  <si>
+    <t>Swiftness</t>
+  </si>
+  <si>
+    <t>Determination</t>
+  </si>
+  <si>
+    <t>Block 5</t>
+  </si>
+  <si>
+    <t>Crystalize</t>
+  </si>
+  <si>
+    <t>When you play this, also pay one mana of a basic color. Gain a crystal of that color to your Inventory.</t>
+  </si>
+  <si>
+    <t>Gain a crystal of any color to your Inventory.</t>
+  </si>
+  <si>
+    <t>Stamina</t>
+  </si>
+  <si>
+    <t>Improvisation</t>
+  </si>
+  <si>
+    <t>Discard another card from your hand to get Move 5, Influence 5, Attack 5 or Block 5.</t>
+  </si>
+  <si>
+    <t>Discard another card from your hand to get Move 3, Influence 3, Attack 3 or Block 3.</t>
+  </si>
+  <si>
+    <t>Threaten</t>
+  </si>
+  <si>
+    <t>Influence 5.
+Reputaion -1.</t>
+  </si>
+  <si>
+    <t>ba5561</t>
+  </si>
+  <si>
+    <t>Undead Horde</t>
+  </si>
+  <si>
+    <t>Rage</t>
+  </si>
+  <si>
+    <t>Attack 4</t>
+  </si>
+  <si>
+    <t>Mage Knight</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>40422e</t>
+  </si>
+  <si>
+    <t>Hidden River</t>
+  </si>
+  <si>
+    <t>Move 2. Move cost of a single Forest is reduced by 2 to a minimum of 1. If you move through two Forests this turn, gain a blue mana token.</t>
+  </si>
+  <si>
+    <t>Move 4. Move cost of a single Forest is reduced by 2 to a minimum of 1. If you move through two Forests this turn, gain a blue Crystal.</t>
+  </si>
+  <si>
+    <t>bfc394
+187cd2</t>
+  </si>
+  <si>
+    <t>71a74a
+c48176</t>
+  </si>
+  <si>
+    <t>3cfeb6
+98441e
+63076d</t>
+  </si>
+  <si>
+    <t>9a67a9
+124af4</t>
+  </si>
+  <si>
+    <t>1a5a80</t>
+  </si>
+  <si>
+    <t>Duscenia</t>
+  </si>
+  <si>
+    <t>Play 2 Wounds as sideways cards for increasing the total effect by 1 then throe away one of those wounds, Heal 2 (1 Heal may be used on your Discard Pile), or gain a green crystal.</t>
+  </si>
+  <si>
+    <t>Play 1 Wound as a sideways card for double the effect then discard it, Heal 1 (may be used on your Discard Pile), or gain a green mana token.</t>
+  </si>
+  <si>
+    <t>29fa1e
+92aed4
+4c5881
+d890d8</t>
+  </si>
+  <si>
+    <t>0cdfcd
+2c15ec
+d90f22
+64b818</t>
+  </si>
+  <si>
+    <t>42adeb</t>
+  </si>
+  <si>
+    <t>Promise</t>
+  </si>
+  <si>
+    <t>d619c6
+bbd990</t>
+  </si>
+  <si>
+    <t>c4ea63
+690015</t>
+  </si>
+  <si>
+    <t>4a2863
+5c9d35</t>
+  </si>
+  <si>
+    <t>1c58fe
+731725
+78d7fc</t>
   </si>
 </sst>
 </file>
@@ -4134,7 +4418,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -4208,6 +4492,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4226,9 +4519,6 @@
     <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4238,10 +4528,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4547,24 +4834,355 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38EE428A-3648-43AA-871D-84443E02FB62}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr defaultColWidth="21.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="21.88671875" style="24"/>
+    <col min="2" max="2" width="7" style="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5546875" style="24" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.44140625" style="24" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="56" style="24" customWidth="1"/>
+    <col min="7" max="16384" width="21.88671875" style="24"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="18" t="s">
+        <v>1186</v>
+      </c>
+      <c r="B1" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="C1" s="19" t="s">
         <v>705</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="D1" s="19" t="s">
         <v>706</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="E1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="F1" s="18" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="14" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>1156</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>1157</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>1158</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>1159</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="14" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>1160</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>1161</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>1162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="14" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>1200</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>1163</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>946</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>1164</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="14" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>1204</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>1167</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>1168</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>1169</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="14" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>1201</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>1170</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>946</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>1090</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="14" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>1192</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>1171</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>941</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>1172</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="14" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>1173</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>1174</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>1175</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="14" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>1194</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>1176</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>946</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>1164</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="14" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>1205</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>1177</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>1179</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>1178</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="14" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>1206</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>1180</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>945</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>1181</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="14" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>1207</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>1184</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>941</v>
+      </c>
+      <c r="F12" s="14" t="s">
+        <v>1185</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="14" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>1202</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>1203</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>945</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="14"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="14" t="s">
+        <v>1166</v>
+      </c>
+      <c r="B15" s="14">
+        <v>585526</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>1165</v>
+      </c>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="14" t="s">
+        <v>1166</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>1182</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>1183</v>
+      </c>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+    </row>
+    <row r="17" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="14" t="s">
+        <v>1197</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>1188</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>1189</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>1190</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>1191</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A18" s="14" t="s">
+        <v>1197</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>1196</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>1199</v>
+      </c>
+      <c r="F18" s="14" t="s">
+        <v>1198</v>
       </c>
     </row>
   </sheetData>
@@ -5498,391 +6116,515 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4487065-31BB-45F2-B223-F2A0D1499038}">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultColWidth="61.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="61.88671875" style="23"/>
-    <col min="5" max="5" width="52.33203125" style="23" customWidth="1"/>
-    <col min="6" max="16384" width="61.88671875" style="1"/>
+    <col min="1" max="1" width="14.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="61.88671875" style="23"/>
+    <col min="6" max="6" width="52.33203125" style="23" customWidth="1"/>
+    <col min="7" max="16384" width="61.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:6" s="2" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="C1" s="19" t="s">
         <v>705</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="D1" s="19" t="s">
         <v>791</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="E1" s="19" t="s">
         <v>822</v>
       </c>
-      <c r="E1" s="19" t="s">
+      <c r="F1" s="19" t="s">
         <v>792</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>1108</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>788</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>789</v>
+      </c>
+      <c r="F2" s="21" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>1109</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>795</v>
+      </c>
+      <c r="E3" s="21" t="s">
+        <v>793</v>
+      </c>
+      <c r="F3" s="21" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>1101</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>798</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>796</v>
+      </c>
+      <c r="F4" s="21" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>1112</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>799</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>820</v>
+      </c>
+      <c r="F5" s="22" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>1104</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>800</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>823</v>
+      </c>
+      <c r="F6" s="21" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>1102</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>801</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>825</v>
+      </c>
+      <c r="F7" s="21" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>1106</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>802</v>
+      </c>
+      <c r="E8" s="21" t="s">
+        <v>827</v>
+      </c>
+      <c r="F8" s="21" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>1116</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>803</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>829</v>
+      </c>
+      <c r="F9" s="21" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>1113</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>804</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>831</v>
+      </c>
+      <c r="F10" s="21" t="s">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>1114</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>805</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>833</v>
+      </c>
+      <c r="F11" s="21" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>1110</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>806</v>
+      </c>
+      <c r="E12" s="21" t="s">
+        <v>835</v>
+      </c>
+      <c r="F12" s="21" t="s">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>1103</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>807</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>836</v>
+      </c>
+      <c r="F13" s="21" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>1100</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>808</v>
+      </c>
+      <c r="E14" s="21" t="s">
+        <v>838</v>
+      </c>
+      <c r="F14" s="21" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="A15" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>809</v>
+      </c>
+      <c r="E15" s="21" t="s">
+        <v>840</v>
+      </c>
+      <c r="F15" s="21" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="C16" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>810</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>842</v>
+      </c>
+      <c r="F16" s="21" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>1107</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>811</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>844</v>
+      </c>
+      <c r="F17" s="21" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>1118</v>
+      </c>
+      <c r="C18" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>788</v>
-      </c>
-      <c r="D2" s="21" t="s">
-        <v>789</v>
-      </c>
-      <c r="E2" s="21" t="s">
-        <v>790</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
-        <v>1116</v>
-      </c>
-      <c r="B3" s="13" t="s">
+      <c r="D18" s="6" t="s">
+        <v>812</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>846</v>
+      </c>
+      <c r="F18" s="21" t="s">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>1117</v>
+      </c>
+      <c r="C19" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>795</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>793</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>794</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
-        <v>1108</v>
-      </c>
-      <c r="B4" s="13" t="s">
+      <c r="D19" s="6" t="s">
+        <v>813</v>
+      </c>
+      <c r="E19" s="21" t="s">
+        <v>848</v>
+      </c>
+      <c r="F19" s="21" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C20" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>798</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>796</v>
-      </c>
-      <c r="E4" s="21" t="s">
-        <v>797</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="6"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="6" t="s">
-        <v>799</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>820</v>
-      </c>
-      <c r="E5" s="22" t="s">
-        <v>821</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
-        <v>1111</v>
-      </c>
-      <c r="B6" s="13" t="s">
+      <c r="D20" s="6" t="s">
+        <v>814</v>
+      </c>
+      <c r="E20" s="21" t="s">
+        <v>850</v>
+      </c>
+      <c r="F20" s="21" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A21" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>1120</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>815</v>
+      </c>
+      <c r="E21" s="21" t="s">
+        <v>852</v>
+      </c>
+      <c r="F21" s="21" t="s">
+        <v>853</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A22" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>1124</v>
+      </c>
+      <c r="C22" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>800</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>823</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>824</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
-        <v>1109</v>
-      </c>
-      <c r="B7" s="13" t="s">
+      <c r="D22" s="6" t="s">
+        <v>816</v>
+      </c>
+      <c r="E22" s="21" t="s">
+        <v>854</v>
+      </c>
+      <c r="F22" s="21" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>1122</v>
+      </c>
+      <c r="C23" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>801</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>825</v>
-      </c>
-      <c r="E7" s="21" t="s">
-        <v>826</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
-        <v>1113</v>
-      </c>
-      <c r="B8" s="13" t="s">
+      <c r="D23" s="6" t="s">
+        <v>817</v>
+      </c>
+      <c r="E23" s="23" t="s">
+        <v>856</v>
+      </c>
+      <c r="F23" s="21" t="s">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>1121</v>
+      </c>
+      <c r="C24" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>802</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>827</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>828</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="6"/>
-      <c r="B9" s="13"/>
-      <c r="C9" s="6" t="s">
-        <v>803</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>829</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>830</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="6"/>
-      <c r="B10" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>804</v>
-      </c>
-      <c r="D10" s="21" t="s">
-        <v>831</v>
-      </c>
-      <c r="E10" s="21" t="s">
-        <v>832</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="6"/>
-      <c r="B11" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>805</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>833</v>
-      </c>
-      <c r="E11" s="21" t="s">
-        <v>834</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
-        <v>1117</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>806</v>
-      </c>
-      <c r="D12" s="21" t="s">
-        <v>835</v>
-      </c>
-      <c r="E12" s="21" t="s">
-        <v>1118</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
-        <v>1110</v>
-      </c>
-      <c r="B13" s="13" t="s">
+      <c r="D24" s="6" t="s">
+        <v>818</v>
+      </c>
+      <c r="E24" s="21" t="s">
+        <v>858</v>
+      </c>
+      <c r="F24" s="21" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C25" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>807</v>
-      </c>
-      <c r="D13" s="21" t="s">
-        <v>836</v>
-      </c>
-      <c r="E13" s="21" t="s">
-        <v>837</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="6" t="s">
-        <v>1107</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>808</v>
-      </c>
-      <c r="D14" s="21" t="s">
-        <v>838</v>
-      </c>
-      <c r="E14" s="21" t="s">
-        <v>839</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
-        <v>1112</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>809</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>840</v>
-      </c>
-      <c r="E15" s="21" t="s">
-        <v>841</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="6"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="6" t="s">
-        <v>810</v>
-      </c>
-      <c r="D16" s="21" t="s">
-        <v>842</v>
-      </c>
-      <c r="E16" s="21" t="s">
-        <v>843</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="6" t="s">
-        <v>1114</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>811</v>
-      </c>
-      <c r="D17" s="21" t="s">
-        <v>844</v>
-      </c>
-      <c r="E17" s="21" t="s">
-        <v>845</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="6"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="6" t="s">
-        <v>812</v>
-      </c>
-      <c r="D18" s="21" t="s">
-        <v>846</v>
-      </c>
-      <c r="E18" s="21" t="s">
-        <v>847</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="6"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="6" t="s">
-        <v>813</v>
-      </c>
-      <c r="D19" s="21" t="s">
-        <v>848</v>
-      </c>
-      <c r="E19" s="21" t="s">
-        <v>849</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="6"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="6" t="s">
-        <v>814</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>850</v>
-      </c>
-      <c r="E20" s="21" t="s">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A21" s="6"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="6" t="s">
-        <v>815</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>852</v>
-      </c>
-      <c r="E21" s="21" t="s">
-        <v>853</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="6"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="6" t="s">
-        <v>816</v>
-      </c>
-      <c r="D22" s="21" t="s">
-        <v>854</v>
-      </c>
-      <c r="E22" s="21" t="s">
-        <v>855</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="6"/>
-      <c r="B23" s="13"/>
-      <c r="C23" s="6" t="s">
-        <v>817</v>
-      </c>
-      <c r="D23" s="23" t="s">
-        <v>856</v>
-      </c>
-      <c r="E23" s="21" t="s">
-        <v>857</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="6"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="6" t="s">
-        <v>818</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>858</v>
-      </c>
-      <c r="E24" s="21" t="s">
-        <v>859</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A25" s="6"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="6" t="s">
+      <c r="D25" s="6" t="s">
         <v>819</v>
       </c>
-      <c r="D25" s="21" t="s">
+      <c r="E25" s="21" t="s">
         <v>860</v>
       </c>
-      <c r="E25" s="21" t="s">
+      <c r="F25" s="21" t="s">
         <v>861</v>
       </c>
     </row>
@@ -5893,329 +6635,456 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1518E3E-453A-4819-AA88-E10B951A9C6F}">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.33203125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="40.88671875" style="3" customWidth="1"/>
-    <col min="5" max="16384" width="9.109375" style="3"/>
+    <col min="1" max="1" width="14.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="24" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:5" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="C1" s="19" t="s">
         <v>791</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="D1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="E1" s="19" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12" t="s">
+    <row r="2" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A2" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="37" t="s">
+        <v>1147</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>863</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="D2" s="12" t="s">
         <v>888</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="E2" s="12" t="s">
         <v>889</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12" t="s">
+    <row r="3" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A3" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="37" t="s">
+        <v>1149</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>864</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="D3" s="12" t="s">
         <v>890</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="E3" s="12" t="s">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="37" t="s">
+        <v>1148</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>865</v>
+      </c>
+      <c r="D4" s="12" t="s">
         <v>891</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="12"/>
-      <c r="B4" s="12" t="s">
-        <v>865</v>
-      </c>
-      <c r="C4" s="12" t="s">
+      <c r="E4" s="12" t="s">
         <v>892</v>
       </c>
-      <c r="D4" s="12" t="s">
+    </row>
+    <row r="5" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="37" t="s">
+        <v>1151</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>866</v>
+      </c>
+      <c r="D5" s="12" t="s">
         <v>893</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="12"/>
-      <c r="B5" s="12" t="s">
-        <v>866</v>
-      </c>
-      <c r="C5" s="12" t="s">
+      <c r="E5" s="12" t="s">
         <v>894</v>
       </c>
-      <c r="D5" s="12" t="s">
+    </row>
+    <row r="6" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="37" t="s">
+        <v>1153</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>867</v>
+      </c>
+      <c r="D6" s="12" t="s">
         <v>895</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="12"/>
-      <c r="B6" s="12" t="s">
-        <v>867</v>
-      </c>
-      <c r="C6" s="12" t="s">
+      <c r="E6" s="12" t="s">
         <v>896</v>
       </c>
-      <c r="D6" s="12" t="s">
+    </row>
+    <row r="7" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="37" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>868</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>897</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="12"/>
-      <c r="B7" s="12" t="s">
-        <v>868</v>
-      </c>
-      <c r="C7" s="12" t="s">
+      <c r="E7" s="12" t="s">
         <v>898</v>
       </c>
-      <c r="D7" s="12" t="s">
+    </row>
+    <row r="8" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>1155</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>869</v>
+      </c>
+      <c r="D8" s="12" t="s">
         <v>899</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12" t="s">
-        <v>869</v>
-      </c>
-      <c r="C8" s="12" t="s">
+      <c r="E8" s="12" t="s">
         <v>900</v>
       </c>
-      <c r="D8" s="12" t="s">
+    </row>
+    <row r="9" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="37" t="s">
+        <v>1154</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>870</v>
+      </c>
+      <c r="D9" s="12" t="s">
         <v>901</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12" t="s">
-        <v>870</v>
-      </c>
-      <c r="C9" s="12" t="s">
+      <c r="E9" s="12" t="s">
         <v>902</v>
       </c>
-      <c r="D9" s="12" t="s">
+    </row>
+    <row r="10" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A10" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="37" t="s">
+        <v>1141</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>871</v>
+      </c>
+      <c r="D10" s="12" t="s">
         <v>903</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="12"/>
-      <c r="B10" s="12" t="s">
-        <v>871</v>
-      </c>
-      <c r="C10" s="12" t="s">
+      <c r="E10" s="12" t="s">
         <v>904</v>
       </c>
-      <c r="D10" s="12" t="s">
+    </row>
+    <row r="11" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A11" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="37" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>872</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>1139</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="37" t="s">
+        <v>1137</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>873</v>
+      </c>
+      <c r="D12" s="12" t="s">
         <v>905</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12" t="s">
-        <v>872</v>
-      </c>
-      <c r="C11" s="12" t="s">
+      <c r="E12" s="12" t="s">
         <v>906</v>
       </c>
-      <c r="D11" s="12" t="s">
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>1142</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>874</v>
+      </c>
+      <c r="D13" s="12" t="s">
         <v>907</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="12"/>
-      <c r="B12" s="12" t="s">
-        <v>873</v>
-      </c>
-      <c r="C12" s="12" t="s">
+      <c r="E13" s="12" t="s">
         <v>908</v>
       </c>
-      <c r="D12" s="12" t="s">
+    </row>
+    <row r="14" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A14" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="37" t="s">
+        <v>1145</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>875</v>
+      </c>
+      <c r="D14" s="12" t="s">
         <v>909</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12" t="s">
-        <v>874</v>
-      </c>
-      <c r="C13" s="12" t="s">
+      <c r="E14" s="12" t="s">
         <v>910</v>
       </c>
-      <c r="D13" s="12" t="s">
+    </row>
+    <row r="15" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A15" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="37" t="s">
+        <v>1146</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>876</v>
+      </c>
+      <c r="D15" s="12" t="s">
         <v>911</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="12"/>
-      <c r="B14" s="12" t="s">
-        <v>875</v>
-      </c>
-      <c r="C14" s="12" t="s">
+      <c r="E15" s="12" t="s">
         <v>912</v>
       </c>
-      <c r="D14" s="12" t="s">
+    </row>
+    <row r="16" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>1143</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>877</v>
+      </c>
+      <c r="D16" s="12" t="s">
         <v>913</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A15" s="12"/>
-      <c r="B15" s="12" t="s">
-        <v>876</v>
-      </c>
-      <c r="C15" s="12" t="s">
+      <c r="E16" s="12" t="s">
         <v>914</v>
       </c>
-      <c r="D15" s="12" t="s">
+    </row>
+    <row r="17" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A17" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="37" t="s">
+        <v>1144</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>878</v>
+      </c>
+      <c r="D17" s="12" t="s">
         <v>915</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="12"/>
-      <c r="B16" s="12" t="s">
-        <v>877</v>
-      </c>
-      <c r="C16" s="12" t="s">
+      <c r="E17" s="12" t="s">
         <v>916</v>
       </c>
-      <c r="D16" s="12" t="s">
+    </row>
+    <row r="18" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A18" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="37" t="s">
+        <v>1132</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>879</v>
+      </c>
+      <c r="D18" s="12" t="s">
         <v>917</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12" t="s">
-        <v>878</v>
-      </c>
-      <c r="C17" s="12" t="s">
+      <c r="E18" s="12" t="s">
         <v>918</v>
       </c>
-      <c r="D17" s="12" t="s">
+    </row>
+    <row r="19" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>1128</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>880</v>
+      </c>
+      <c r="D19" s="12" t="s">
         <v>919</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12" t="s">
-        <v>879</v>
-      </c>
-      <c r="C18" s="12" t="s">
+      <c r="E19" s="12" t="s">
         <v>920</v>
       </c>
-      <c r="D18" s="12" t="s">
+    </row>
+    <row r="20" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A20" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>1125</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>881</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>1126</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>1127</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" s="37" t="s">
+        <v>1133</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>882</v>
+      </c>
+      <c r="D21" s="12" t="s">
         <v>921</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12" t="s">
-        <v>880</v>
-      </c>
-      <c r="C19" s="12" t="s">
+      <c r="E21" s="12" t="s">
         <v>922</v>
       </c>
-      <c r="D19" s="12" t="s">
+    </row>
+    <row r="22" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="37" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>883</v>
+      </c>
+      <c r="D22" s="12" t="s">
         <v>923</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12" t="s">
-        <v>881</v>
-      </c>
-      <c r="C20" s="12" t="s">
+      <c r="E22" s="12" t="s">
         <v>924</v>
       </c>
-      <c r="D20" s="12" t="s">
+    </row>
+    <row r="23" spans="1:5" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A23" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="25" t="s">
+        <v>1130</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>884</v>
+      </c>
+      <c r="D23" s="12" t="s">
         <v>925</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12" t="s">
-        <v>882</v>
-      </c>
-      <c r="C21" s="12" t="s">
+      <c r="E23" s="12" t="s">
         <v>926</v>
       </c>
-      <c r="D21" s="12" t="s">
+    </row>
+    <row r="24" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="A24" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" s="37" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>885</v>
+      </c>
+      <c r="D24" s="12" t="s">
         <v>927</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="12"/>
-      <c r="B22" s="12" t="s">
-        <v>883</v>
-      </c>
-      <c r="C22" s="12" t="s">
+      <c r="E24" s="12" t="s">
         <v>928</v>
       </c>
-      <c r="D22" s="12" t="s">
+    </row>
+    <row r="25" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="25" t="s">
+        <v>1129</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>886</v>
+      </c>
+      <c r="D25" s="12" t="s">
         <v>929</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="12"/>
-      <c r="B23" s="12" t="s">
-        <v>884</v>
-      </c>
-      <c r="C23" s="12" t="s">
+      <c r="E25" s="12" t="s">
         <v>930</v>
       </c>
-      <c r="D23" s="12" t="s">
-        <v>931</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A24" s="12"/>
-      <c r="B24" s="12" t="s">
-        <v>885</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>932</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>933</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12" t="s">
-        <v>886</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>934</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>935</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A26" s="12"/>
-      <c r="B26" s="12" t="s">
+    </row>
+    <row r="26" spans="1:5" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" s="37" t="s">
+        <v>1135</v>
+      </c>
+      <c r="C26" s="12" t="s">
         <v>887</v>
       </c>
-      <c r="C26" s="12" t="s">
-        <v>936</v>
-      </c>
       <c r="D26" s="12" t="s">
-        <v>937</v>
-      </c>
+        <v>1136</v>
+      </c>
+      <c r="E26" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6254,74 +7123,74 @@
         <v>706</v>
       </c>
       <c r="C1" s="19" t="s">
-        <v>993</v>
+        <v>986</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>994</v>
+        <v>987</v>
       </c>
       <c r="E1" s="19" t="s">
-        <v>995</v>
+        <v>988</v>
       </c>
       <c r="F1" s="19" t="s">
-        <v>999</v>
+        <v>992</v>
       </c>
       <c r="G1" s="19" t="s">
-        <v>996</v>
+        <v>989</v>
       </c>
       <c r="H1" s="18" t="s">
-        <v>954</v>
+        <v>947</v>
       </c>
       <c r="I1" s="18" t="s">
+        <v>942</v>
+      </c>
+      <c r="J1" s="18" t="s">
+        <v>948</v>
+      </c>
+      <c r="K1" s="18" t="s">
+        <v>943</v>
+      </c>
+      <c r="L1" s="18" t="s">
         <v>949</v>
       </c>
-      <c r="J1" s="18" t="s">
-        <v>955</v>
-      </c>
-      <c r="K1" s="18" t="s">
-        <v>950</v>
-      </c>
-      <c r="L1" s="18" t="s">
-        <v>956</v>
-      </c>
       <c r="M1" s="18" t="s">
-        <v>951</v>
+        <v>944</v>
       </c>
       <c r="N1" s="18" t="s">
-        <v>1042</v>
+        <v>1035</v>
       </c>
       <c r="O1" s="18" t="s">
-        <v>1043</v>
+        <v>1036</v>
       </c>
       <c r="P1" s="18" t="s">
-        <v>1047</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A2" s="35" t="s">
-        <v>938</v>
-      </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="35"/>
-      <c r="J2" s="35"/>
-      <c r="K2" s="35"/>
-      <c r="L2" s="35"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="35"/>
-      <c r="O2" s="35"/>
-      <c r="P2" s="35"/>
+      <c r="A2" s="26" t="s">
+        <v>931</v>
+      </c>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
+      <c r="P2" s="26"/>
     </row>
     <row r="3" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
-        <v>1024</v>
+        <v>1017</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>980</v>
+        <v>973</v>
       </c>
       <c r="C3" s="14">
         <v>1</v>
@@ -6334,19 +7203,19 @@
       </c>
       <c r="F3" s="14"/>
       <c r="G3" s="14" t="s">
-        <v>1002</v>
+        <v>995</v>
       </c>
       <c r="H3" s="14"/>
       <c r="I3" s="12" t="s">
-        <v>948</v>
+        <v>941</v>
       </c>
       <c r="J3" s="14"/>
       <c r="K3" s="12" t="s">
-        <v>952</v>
+        <v>945</v>
       </c>
       <c r="L3" s="14"/>
       <c r="M3" s="12" t="s">
-        <v>953</v>
+        <v>946</v>
       </c>
       <c r="N3" s="12"/>
       <c r="O3" s="12"/>
@@ -6354,10 +7223,10 @@
     </row>
     <row r="4" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
-        <v>1011</v>
+        <v>1004</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>979</v>
+        <v>972</v>
       </c>
       <c r="C4" s="14">
         <v>1</v>
@@ -6370,21 +7239,21 @@
       </c>
       <c r="F4" s="14"/>
       <c r="G4" s="14" t="s">
-        <v>997</v>
+        <v>990</v>
       </c>
       <c r="H4" s="14" t="s">
-        <v>990</v>
+        <v>983</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>989</v>
+        <v>982</v>
       </c>
       <c r="J4" s="14"/>
       <c r="K4" s="12" t="s">
-        <v>957</v>
+        <v>950</v>
       </c>
       <c r="L4" s="14"/>
       <c r="M4" s="12" t="s">
-        <v>958</v>
+        <v>951</v>
       </c>
       <c r="N4" s="12"/>
       <c r="O4" s="12"/>
@@ -6392,10 +7261,10 @@
     </row>
     <row r="5" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
-        <v>1009</v>
+        <v>1002</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>978</v>
+        <v>971</v>
       </c>
       <c r="C5" s="14">
         <v>1</v>
@@ -6408,15 +7277,15 @@
       </c>
       <c r="F5" s="14"/>
       <c r="G5" s="14" t="s">
-        <v>1002</v>
+        <v>995</v>
       </c>
       <c r="H5" s="14"/>
       <c r="I5" s="12" t="s">
-        <v>984</v>
+        <v>977</v>
       </c>
       <c r="J5" s="14"/>
       <c r="K5" s="12" t="s">
-        <v>983</v>
+        <v>976</v>
       </c>
       <c r="L5" s="14"/>
       <c r="M5" s="12"/>
@@ -6426,10 +7295,10 @@
     </row>
     <row r="6" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
-        <v>1008</v>
+        <v>1001</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>977</v>
+        <v>970</v>
       </c>
       <c r="C6" s="14">
         <v>2</v>
@@ -6442,15 +7311,15 @@
       </c>
       <c r="F6" s="14"/>
       <c r="G6" s="14" t="s">
-        <v>1001</v>
+        <v>994</v>
       </c>
       <c r="H6" s="14"/>
       <c r="I6" s="12" t="s">
-        <v>981</v>
+        <v>974</v>
       </c>
       <c r="J6" s="14"/>
       <c r="K6" s="12" t="s">
-        <v>982</v>
+        <v>975</v>
       </c>
       <c r="L6" s="14"/>
       <c r="M6" s="12"/>
@@ -6460,10 +7329,10 @@
     </row>
     <row r="7" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="12" t="s">
-        <v>1010</v>
+        <v>1003</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>976</v>
+        <v>969</v>
       </c>
       <c r="C7" s="14">
         <v>2</v>
@@ -6476,15 +7345,15 @@
       </c>
       <c r="F7" s="14"/>
       <c r="G7" s="14" t="s">
-        <v>1001</v>
+        <v>994</v>
       </c>
       <c r="H7" s="14"/>
       <c r="I7" s="12" t="s">
-        <v>985</v>
+        <v>978</v>
       </c>
       <c r="J7" s="14"/>
       <c r="K7" s="12" t="s">
-        <v>986</v>
+        <v>979</v>
       </c>
       <c r="L7" s="14"/>
       <c r="M7" s="12"/>
@@ -6494,10 +7363,10 @@
     </row>
     <row r="8" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
-        <v>1016</v>
+        <v>1009</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>975</v>
+        <v>968</v>
       </c>
       <c r="C8" s="14">
         <v>2</v>
@@ -6510,15 +7379,15 @@
       </c>
       <c r="F8" s="14"/>
       <c r="G8" s="14" t="s">
-        <v>1014</v>
+        <v>1007</v>
       </c>
       <c r="H8" s="14"/>
       <c r="I8" s="12" t="s">
-        <v>981</v>
+        <v>974</v>
       </c>
       <c r="J8" s="14"/>
       <c r="K8" s="12" t="s">
-        <v>1015</v>
+        <v>1008</v>
       </c>
       <c r="L8" s="14"/>
       <c r="M8" s="12"/>
@@ -6528,10 +7397,10 @@
     </row>
     <row r="9" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
-        <v>1012</v>
+        <v>1005</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>974</v>
+        <v>967</v>
       </c>
       <c r="C9" s="14">
         <v>2</v>
@@ -6543,26 +7412,26 @@
         <v>3</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>1000</v>
+        <v>993</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>998</v>
+        <v>991</v>
       </c>
       <c r="H9" s="14"/>
       <c r="I9" s="12" t="s">
-        <v>948</v>
+        <v>941</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>991</v>
+        <v>984</v>
       </c>
       <c r="K9" s="12" t="s">
-        <v>987</v>
+        <v>980</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="M9" s="12" t="s">
-        <v>988</v>
+        <v>981</v>
       </c>
       <c r="N9" s="12"/>
       <c r="O9" s="12"/>
@@ -6570,10 +7439,10 @@
     </row>
     <row r="10" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="12" t="s">
-        <v>1013</v>
+        <v>1006</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>973</v>
+        <v>966</v>
       </c>
       <c r="C10" s="14">
         <v>2</v>
@@ -6585,35 +7454,35 @@
         <v>2</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>1000</v>
+        <v>993</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>1003</v>
+        <v>996</v>
       </c>
       <c r="H10" s="14"/>
       <c r="I10" s="12" t="s">
-        <v>1004</v>
+        <v>997</v>
       </c>
       <c r="J10" s="14" t="s">
-        <v>1005</v>
+        <v>998</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>1006</v>
+        <v>999</v>
       </c>
       <c r="L10" s="14"/>
       <c r="M10" s="12" t="s">
-        <v>1007</v>
+        <v>1000</v>
       </c>
       <c r="N10" s="12"/>
       <c r="O10" s="12"/>
       <c r="P10" s="12"/>
     </row>
     <row r="11" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="36" t="s">
-        <v>1021</v>
+      <c r="A11" s="25" t="s">
+        <v>1014</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>972</v>
+        <v>965</v>
       </c>
       <c r="C11" s="14">
         <v>2</v>
@@ -6626,17 +7495,17 @@
       </c>
       <c r="F11" s="14"/>
       <c r="G11" s="14" t="s">
-        <v>1018</v>
+        <v>1011</v>
       </c>
       <c r="H11" s="14"/>
       <c r="I11" s="12" t="s">
-        <v>981</v>
+        <v>974</v>
       </c>
       <c r="J11" s="14" t="s">
-        <v>991</v>
+        <v>984</v>
       </c>
       <c r="K11" s="12" t="s">
-        <v>1020</v>
+        <v>1013</v>
       </c>
       <c r="L11" s="14"/>
       <c r="M11" s="12"/>
@@ -6646,10 +7515,10 @@
     </row>
     <row r="12" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
-        <v>1017</v>
+        <v>1010</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>971</v>
+        <v>964</v>
       </c>
       <c r="C12" s="14">
         <v>2</v>
@@ -6662,17 +7531,17 @@
       </c>
       <c r="F12" s="14"/>
       <c r="G12" s="14" t="s">
-        <v>1018</v>
+        <v>1011</v>
       </c>
       <c r="H12" s="14"/>
       <c r="I12" s="12" t="s">
-        <v>981</v>
+        <v>974</v>
       </c>
       <c r="J12" s="14" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="K12" s="12" t="s">
-        <v>1019</v>
+        <v>1012</v>
       </c>
       <c r="L12" s="14"/>
       <c r="M12" s="12"/>
@@ -6682,10 +7551,10 @@
     </row>
     <row r="13" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="12" t="s">
-        <v>1022</v>
+        <v>1015</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>970</v>
+        <v>963</v>
       </c>
       <c r="C13" s="14">
         <v>2</v>
@@ -6698,17 +7567,17 @@
       </c>
       <c r="F13" s="14"/>
       <c r="G13" s="14" t="s">
-        <v>1018</v>
+        <v>1011</v>
       </c>
       <c r="H13" s="14"/>
       <c r="I13" s="12" t="s">
-        <v>981</v>
+        <v>974</v>
       </c>
       <c r="J13" s="14" t="s">
-        <v>990</v>
+        <v>983</v>
       </c>
       <c r="K13" s="12" t="s">
-        <v>1023</v>
+        <v>1016</v>
       </c>
       <c r="L13" s="14"/>
       <c r="M13" s="12"/>
@@ -6718,29 +7587,29 @@
     </row>
     <row r="14" spans="1:16" ht="72" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
-        <v>1044</v>
+        <v>1037</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>969</v>
+        <v>962</v>
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="14"/>
       <c r="E14" s="14"/>
       <c r="F14" s="14"/>
       <c r="G14" s="14" t="s">
-        <v>1036</v>
+        <v>1029</v>
       </c>
       <c r="H14" s="14"/>
       <c r="I14" s="12" t="s">
-        <v>1033</v>
+        <v>1026</v>
       </c>
       <c r="J14" s="14"/>
       <c r="K14" s="12" t="s">
-        <v>1034</v>
+        <v>1027</v>
       </c>
       <c r="L14" s="14"/>
       <c r="M14" s="12" t="s">
-        <v>1035</v>
+        <v>1028</v>
       </c>
       <c r="N14" s="12"/>
       <c r="O14" s="12"/>
@@ -6748,10 +7617,10 @@
     </row>
     <row r="15" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
-        <v>1029</v>
+        <v>1022</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>968</v>
+        <v>961</v>
       </c>
       <c r="C15" s="14">
         <v>1</v>
@@ -6764,19 +7633,19 @@
       </c>
       <c r="F15" s="14"/>
       <c r="G15" s="14" t="s">
-        <v>1030</v>
+        <v>1023</v>
       </c>
       <c r="H15" s="14"/>
       <c r="I15" s="12" t="s">
-        <v>983</v>
+        <v>976</v>
       </c>
       <c r="J15" s="14"/>
       <c r="K15" s="12" t="s">
-        <v>1031</v>
+        <v>1024</v>
       </c>
       <c r="L15" s="14"/>
       <c r="M15" s="12" t="s">
-        <v>1032</v>
+        <v>1025</v>
       </c>
       <c r="N15" s="12"/>
       <c r="O15" s="12"/>
@@ -6784,10 +7653,10 @@
     </row>
     <row r="16" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="12" t="s">
-        <v>1025</v>
+        <v>1018</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>967</v>
+        <v>960</v>
       </c>
       <c r="C16" s="14">
         <v>2</v>
@@ -6800,19 +7669,19 @@
       </c>
       <c r="F16" s="14"/>
       <c r="G16" s="14" t="s">
-        <v>1014</v>
+        <v>1007</v>
       </c>
       <c r="H16" s="14"/>
       <c r="I16" s="12" t="s">
-        <v>1026</v>
+        <v>1019</v>
       </c>
       <c r="J16" s="14"/>
       <c r="K16" s="12" t="s">
-        <v>1027</v>
+        <v>1020</v>
       </c>
       <c r="L16" s="14"/>
       <c r="M16" s="12" t="s">
-        <v>1028</v>
+        <v>1021</v>
       </c>
       <c r="N16" s="12"/>
       <c r="O16" s="12"/>
@@ -6820,10 +7689,10 @@
     </row>
     <row r="17" spans="1:16" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A17" s="12" t="s">
-        <v>1045</v>
+        <v>1038</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>966</v>
+        <v>959</v>
       </c>
       <c r="C17" s="14">
         <v>2</v>
@@ -6836,54 +7705,54 @@
       </c>
       <c r="F17" s="14"/>
       <c r="G17" s="14" t="s">
-        <v>1037</v>
+        <v>1030</v>
       </c>
       <c r="H17" s="14"/>
       <c r="I17" s="12" t="s">
-        <v>1038</v>
+        <v>1031</v>
       </c>
       <c r="J17" s="14"/>
       <c r="K17" s="12" t="s">
-        <v>1039</v>
+        <v>1032</v>
       </c>
       <c r="L17" s="14"/>
       <c r="M17" s="12" t="s">
-        <v>1040</v>
+        <v>1033</v>
       </c>
       <c r="N17" s="12"/>
       <c r="O17" s="12" t="s">
-        <v>1041</v>
+        <v>1034</v>
       </c>
       <c r="P17" s="12" t="s">
-        <v>1046</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A18" s="35" t="s">
-        <v>939</v>
-      </c>
-      <c r="B18" s="35"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="35"/>
-      <c r="G18" s="35"/>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
-      <c r="J18" s="35"/>
-      <c r="K18" s="35"/>
-      <c r="L18" s="35"/>
-      <c r="M18" s="35"/>
-      <c r="N18" s="35"/>
-      <c r="O18" s="35"/>
-      <c r="P18" s="35"/>
+      <c r="A18" s="26" t="s">
+        <v>932</v>
+      </c>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="26"/>
+      <c r="I18" s="26"/>
+      <c r="J18" s="26"/>
+      <c r="K18" s="26"/>
+      <c r="L18" s="26"/>
+      <c r="M18" s="26"/>
+      <c r="N18" s="26"/>
+      <c r="O18" s="26"/>
+      <c r="P18" s="26"/>
     </row>
     <row r="19" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
-        <v>1061</v>
+        <v>1054</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>940</v>
+        <v>933</v>
       </c>
       <c r="C19" s="14">
         <v>3</v>
@@ -6895,20 +7764,20 @@
         <v>4</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>1062</v>
+        <v>1055</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>998</v>
+        <v>991</v>
       </c>
       <c r="H19" s="14"/>
       <c r="I19" s="12" t="s">
-        <v>981</v>
+        <v>974</v>
       </c>
       <c r="J19" s="14" t="s">
-        <v>991</v>
+        <v>984</v>
       </c>
       <c r="K19" s="12" t="s">
-        <v>1063</v>
+        <v>1056</v>
       </c>
       <c r="L19" s="14"/>
       <c r="M19" s="12"/>
@@ -6918,10 +7787,10 @@
     </row>
     <row r="20" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="12" t="s">
-        <v>1059</v>
+        <v>1052</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>941</v>
+        <v>934</v>
       </c>
       <c r="C20" s="14">
         <v>3</v>
@@ -6933,20 +7802,20 @@
         <v>4</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>1058</v>
+        <v>1051</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>998</v>
+        <v>991</v>
       </c>
       <c r="H20" s="14"/>
       <c r="I20" s="12" t="s">
-        <v>981</v>
+        <v>974</v>
       </c>
       <c r="J20" s="14" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="K20" s="12" t="s">
-        <v>1060</v>
+        <v>1053</v>
       </c>
       <c r="L20" s="14"/>
       <c r="M20" s="12"/>
@@ -6956,10 +7825,10 @@
     </row>
     <row r="21" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="12" t="s">
-        <v>1054</v>
+        <v>1047</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>942</v>
+        <v>935</v>
       </c>
       <c r="C21" s="14">
         <v>3</v>
@@ -6971,24 +7840,24 @@
         <v>4</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>1052</v>
+        <v>1045</v>
       </c>
       <c r="G21" s="14" t="s">
-        <v>1003</v>
+        <v>996</v>
       </c>
       <c r="H21" s="14"/>
       <c r="I21" s="12" t="s">
-        <v>1055</v>
+        <v>1048</v>
       </c>
       <c r="J21" s="14" t="s">
-        <v>991</v>
+        <v>984</v>
       </c>
       <c r="K21" s="21" t="s">
-        <v>1056</v>
+        <v>1049</v>
       </c>
       <c r="L21" s="14"/>
       <c r="M21" s="12" t="s">
-        <v>1057</v>
+        <v>1050</v>
       </c>
       <c r="N21" s="12"/>
       <c r="O21" s="12"/>
@@ -6996,10 +7865,10 @@
     </row>
     <row r="22" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="12" t="s">
-        <v>1064</v>
+        <v>1057</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="C22" s="14">
         <v>3</v>
@@ -7011,24 +7880,24 @@
         <v>4</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>1053</v>
+        <v>1046</v>
       </c>
       <c r="G22" s="14" t="s">
-        <v>1003</v>
+        <v>996</v>
       </c>
       <c r="H22" s="14"/>
       <c r="I22" s="12" t="s">
-        <v>1065</v>
+        <v>1058</v>
       </c>
       <c r="J22" s="14" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="K22" s="21" t="s">
-        <v>1066</v>
+        <v>1059</v>
       </c>
       <c r="L22" s="14"/>
       <c r="M22" s="12" t="s">
-        <v>1067</v>
+        <v>1060</v>
       </c>
       <c r="N22" s="12"/>
       <c r="O22" s="12"/>
@@ -7036,10 +7905,10 @@
     </row>
     <row r="23" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
-        <v>1068</v>
+        <v>1061</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>944</v>
+        <v>937</v>
       </c>
       <c r="C23" s="14">
         <v>3</v>
@@ -7052,17 +7921,17 @@
       </c>
       <c r="F23" s="14"/>
       <c r="G23" s="14" t="s">
-        <v>1049</v>
+        <v>1042</v>
       </c>
       <c r="H23" s="14"/>
       <c r="I23" s="12" t="s">
-        <v>1050</v>
+        <v>1043</v>
       </c>
       <c r="J23" s="14" t="s">
-        <v>991</v>
+        <v>984</v>
       </c>
       <c r="K23" s="12" t="s">
-        <v>1069</v>
+        <v>1062</v>
       </c>
       <c r="L23" s="14"/>
       <c r="M23" s="12"/>
@@ -7072,10 +7941,10 @@
     </row>
     <row r="24" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="12" t="s">
-        <v>1048</v>
+        <v>1041</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>945</v>
+        <v>938</v>
       </c>
       <c r="C24" s="14">
         <v>3</v>
@@ -7088,17 +7957,17 @@
       </c>
       <c r="F24" s="14"/>
       <c r="G24" s="14" t="s">
-        <v>1049</v>
+        <v>1042</v>
       </c>
       <c r="H24" s="14"/>
       <c r="I24" s="12" t="s">
-        <v>1050</v>
+        <v>1043</v>
       </c>
       <c r="J24" s="14" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="K24" s="12" t="s">
-        <v>1051</v>
+        <v>1044</v>
       </c>
       <c r="L24" s="14"/>
       <c r="M24" s="12"/>
@@ -7108,10 +7977,10 @@
     </row>
     <row r="25" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
-        <v>1081</v>
+        <v>1074</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>965</v>
+        <v>958</v>
       </c>
       <c r="C25" s="14">
         <v>3</v>
@@ -7126,19 +7995,19 @@
       <c r="G25" s="14"/>
       <c r="H25" s="14"/>
       <c r="I25" s="21" t="s">
-        <v>1082</v>
+        <v>1075</v>
       </c>
       <c r="J25" s="14" t="s">
-        <v>991</v>
+        <v>984</v>
       </c>
       <c r="K25" s="21" t="s">
-        <v>1083</v>
+        <v>1076</v>
       </c>
       <c r="L25" s="14" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="M25" s="21" t="s">
-        <v>1084</v>
+        <v>1077</v>
       </c>
       <c r="N25" s="12"/>
       <c r="O25" s="12"/>
@@ -7146,10 +8015,10 @@
     </row>
     <row r="26" spans="1:16" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
-        <v>1070</v>
+        <v>1063</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>946</v>
+        <v>939</v>
       </c>
       <c r="C26" s="14">
         <v>4</v>
@@ -7161,24 +8030,24 @@
         <v>5</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>1071</v>
+        <v>1064</v>
       </c>
       <c r="G26" s="14" t="s">
-        <v>1072</v>
+        <v>1065</v>
       </c>
       <c r="H26" s="14"/>
       <c r="I26" s="12" t="s">
-        <v>1073</v>
+        <v>1066</v>
       </c>
       <c r="J26" s="14"/>
       <c r="K26" s="12" t="s">
-        <v>1074</v>
+        <v>1067</v>
       </c>
       <c r="L26" s="14" t="s">
-        <v>1076</v>
+        <v>1069</v>
       </c>
       <c r="M26" s="12" t="s">
-        <v>1075</v>
+        <v>1068</v>
       </c>
       <c r="N26" s="12"/>
       <c r="O26" s="12"/>
@@ -7186,10 +8055,10 @@
     </row>
     <row r="27" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A27" s="12" t="s">
-        <v>1077</v>
+        <v>1070</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>947</v>
+        <v>940</v>
       </c>
       <c r="C27" s="14">
         <v>4</v>
@@ -7202,21 +8071,21 @@
       </c>
       <c r="F27" s="14"/>
       <c r="G27" s="14" t="s">
-        <v>1072</v>
+        <v>1065</v>
       </c>
       <c r="H27" s="14"/>
       <c r="I27" s="12" t="s">
-        <v>1078</v>
+        <v>1071</v>
       </c>
       <c r="J27" s="14"/>
       <c r="K27" s="12" t="s">
-        <v>1079</v>
+        <v>1072</v>
       </c>
       <c r="L27" s="14" t="s">
-        <v>990</v>
+        <v>983</v>
       </c>
       <c r="M27" s="12" t="s">
-        <v>1080</v>
+        <v>1073</v>
       </c>
       <c r="N27" s="12"/>
       <c r="O27" s="12"/>
@@ -7224,10 +8093,10 @@
     </row>
     <row r="28" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A28" s="12" t="s">
-        <v>1092</v>
+        <v>1085</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>964</v>
+        <v>957</v>
       </c>
       <c r="C28" s="14">
         <v>3</v>
@@ -7240,21 +8109,21 @@
       </c>
       <c r="F28" s="14"/>
       <c r="G28" s="14" t="s">
-        <v>1085</v>
+        <v>1078</v>
       </c>
       <c r="H28" s="14"/>
       <c r="I28" s="12" t="s">
-        <v>1050</v>
+        <v>1043</v>
       </c>
       <c r="J28" s="14" t="s">
-        <v>1005</v>
+        <v>998</v>
       </c>
       <c r="K28" s="12" t="s">
-        <v>1093</v>
+        <v>1086</v>
       </c>
       <c r="L28" s="14"/>
       <c r="M28" s="12" t="s">
-        <v>1087</v>
+        <v>1080</v>
       </c>
       <c r="N28" s="12"/>
       <c r="O28" s="12"/>
@@ -7262,10 +8131,10 @@
     </row>
     <row r="29" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A29" s="12" t="s">
-        <v>1090</v>
+        <v>1083</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>963</v>
+        <v>956</v>
       </c>
       <c r="C29" s="14">
         <v>3</v>
@@ -7277,24 +8146,24 @@
         <v>3</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>1000</v>
+        <v>993</v>
       </c>
       <c r="G29" s="14" t="s">
-        <v>1085</v>
+        <v>1078</v>
       </c>
       <c r="H29" s="14"/>
       <c r="I29" s="12" t="s">
-        <v>1050</v>
+        <v>1043</v>
       </c>
       <c r="J29" s="14" t="s">
-        <v>990</v>
+        <v>983</v>
       </c>
       <c r="K29" s="12" t="s">
-        <v>1091</v>
+        <v>1084</v>
       </c>
       <c r="L29" s="14"/>
       <c r="M29" s="12" t="s">
-        <v>1087</v>
+        <v>1080</v>
       </c>
       <c r="N29" s="12"/>
       <c r="O29" s="12"/>
@@ -7302,10 +8171,10 @@
     </row>
     <row r="30" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A30" s="12" t="s">
-        <v>1089</v>
+        <v>1082</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>962</v>
+        <v>955</v>
       </c>
       <c r="C30" s="14">
         <v>3</v>
@@ -7317,37 +8186,37 @@
         <v>4</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>1053</v>
+        <v>1046</v>
       </c>
       <c r="G30" s="14" t="s">
-        <v>1085</v>
+        <v>1078</v>
       </c>
       <c r="H30" s="14"/>
       <c r="I30" s="12" t="s">
-        <v>1050</v>
+        <v>1043</v>
       </c>
       <c r="J30" s="14" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="K30" s="12" t="s">
-        <v>1086</v>
+        <v>1079</v>
       </c>
       <c r="L30" s="14"/>
       <c r="M30" s="12" t="s">
-        <v>1087</v>
+        <v>1080</v>
       </c>
       <c r="N30" s="12"/>
       <c r="O30" s="12"/>
       <c r="P30" s="12" t="s">
-        <v>1088</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A31" s="12" t="s">
-        <v>1094</v>
+        <v>1087</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>961</v>
+        <v>954</v>
       </c>
       <c r="C31" s="14">
         <v>3</v>
@@ -7359,24 +8228,24 @@
         <v>4</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>1052</v>
+        <v>1045</v>
       </c>
       <c r="G31" s="14" t="s">
-        <v>1085</v>
+        <v>1078</v>
       </c>
       <c r="H31" s="14"/>
       <c r="I31" s="12" t="s">
-        <v>1050</v>
+        <v>1043</v>
       </c>
       <c r="J31" s="14" t="s">
-        <v>991</v>
+        <v>984</v>
       </c>
       <c r="K31" s="12" t="s">
-        <v>1095</v>
+        <v>1088</v>
       </c>
       <c r="L31" s="14"/>
       <c r="M31" s="12" t="s">
-        <v>1087</v>
+        <v>1080</v>
       </c>
       <c r="N31" s="12"/>
       <c r="O31" s="12"/>
@@ -7384,10 +8253,10 @@
     </row>
     <row r="32" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A32" s="12" t="s">
-        <v>1096</v>
+        <v>1089</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>960</v>
+        <v>953</v>
       </c>
       <c r="C32" s="14">
         <v>3</v>
@@ -7399,26 +8268,26 @@
         <v>4</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>1071</v>
+        <v>1064</v>
       </c>
       <c r="G32" s="14" t="s">
-        <v>1003</v>
+        <v>996</v>
       </c>
       <c r="H32" s="14"/>
       <c r="I32" s="12" t="s">
-        <v>1097</v>
+        <v>1090</v>
       </c>
       <c r="J32" s="14" t="s">
-        <v>1005</v>
+        <v>998</v>
       </c>
       <c r="K32" s="12" t="s">
-        <v>1098</v>
+        <v>1091</v>
       </c>
       <c r="L32" s="14" t="s">
-        <v>990</v>
+        <v>983</v>
       </c>
       <c r="M32" s="12" t="s">
-        <v>1099</v>
+        <v>1092</v>
       </c>
       <c r="N32" s="12"/>
       <c r="O32" s="12"/>
@@ -7426,10 +8295,10 @@
     </row>
     <row r="33" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="12" t="s">
-        <v>1100</v>
+        <v>1093</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>959</v>
+        <v>952</v>
       </c>
       <c r="C33" s="14">
         <v>4</v>
@@ -7441,37 +8310,37 @@
         <v>3</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>1101</v>
+        <v>1094</v>
       </c>
       <c r="G33" s="14" t="s">
-        <v>1072</v>
+        <v>1065</v>
       </c>
       <c r="H33" s="14" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="I33" s="12" t="s">
-        <v>1102</v>
+        <v>1095</v>
       </c>
       <c r="J33" s="14" t="s">
-        <v>991</v>
+        <v>984</v>
       </c>
       <c r="K33" s="12" t="s">
-        <v>1103</v>
+        <v>1096</v>
       </c>
       <c r="L33" s="14" t="s">
-        <v>990</v>
+        <v>983</v>
       </c>
       <c r="M33" s="12" t="s">
-        <v>1104</v>
+        <v>1097</v>
       </c>
       <c r="N33" s="14" t="s">
-        <v>1005</v>
+        <v>998</v>
       </c>
       <c r="O33" s="12" t="s">
-        <v>1105</v>
+        <v>1098</v>
       </c>
       <c r="P33" s="12" t="s">
-        <v>1106</v>
+        <v>1099</v>
       </c>
     </row>
   </sheetData>
@@ -7510,12 +8379,12 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
     </row>
     <row r="3" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
@@ -7654,12 +8523,12 @@
       <c r="D13" s="6"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="25" t="s">
+      <c r="A14" s="28" t="s">
         <v>124</v>
       </c>
-      <c r="B14" s="26"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="27"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="30"/>
     </row>
     <row r="15" spans="1:4" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
@@ -7798,12 +8667,12 @@
       <c r="D25" s="6"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="25" t="s">
+      <c r="A26" s="28" t="s">
         <v>143</v>
       </c>
-      <c r="B26" s="26"/>
-      <c r="C26" s="26"/>
-      <c r="D26" s="27"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="30"/>
     </row>
     <row r="27" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
@@ -7942,12 +8811,12 @@
       <c r="D37" s="6"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" s="25" t="s">
+      <c r="A38" s="28" t="s">
         <v>163</v>
       </c>
-      <c r="B38" s="26"/>
-      <c r="C38" s="26"/>
-      <c r="D38" s="27"/>
+      <c r="B38" s="29"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="30"/>
     </row>
     <row r="39" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A39" s="9" t="s">
@@ -8086,12 +8955,12 @@
       <c r="D49" s="6"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A50" s="25" t="s">
+      <c r="A50" s="28" t="s">
         <v>184</v>
       </c>
-      <c r="B50" s="26"/>
-      <c r="C50" s="26"/>
-      <c r="D50" s="27"/>
+      <c r="B50" s="29"/>
+      <c r="C50" s="29"/>
+      <c r="D50" s="30"/>
     </row>
     <row r="51" spans="1:4" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A51" s="4">
@@ -8230,12 +9099,12 @@
       <c r="D61" s="6"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A62" s="25" t="s">
+      <c r="A62" s="28" t="s">
         <v>204</v>
       </c>
-      <c r="B62" s="26"/>
-      <c r="C62" s="26"/>
-      <c r="D62" s="27"/>
+      <c r="B62" s="29"/>
+      <c r="C62" s="29"/>
+      <c r="D62" s="30"/>
     </row>
     <row r="63" spans="1:4" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
@@ -8374,12 +9243,12 @@
       <c r="D73" s="6"/>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A74" s="25" t="s">
+      <c r="A74" s="28" t="s">
         <v>225</v>
       </c>
-      <c r="B74" s="26"/>
-      <c r="C74" s="26"/>
-      <c r="D74" s="27"/>
+      <c r="B74" s="29"/>
+      <c r="C74" s="29"/>
+      <c r="D74" s="30"/>
     </row>
     <row r="75" spans="1:4" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A75" s="4">
@@ -8518,12 +9387,12 @@
       <c r="D85" s="6"/>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A86" s="25" t="s">
+      <c r="A86" s="28" t="s">
         <v>379</v>
       </c>
-      <c r="B86" s="26"/>
-      <c r="C86" s="26"/>
-      <c r="D86" s="27"/>
+      <c r="B86" s="29"/>
+      <c r="C86" s="29"/>
+      <c r="D86" s="30"/>
     </row>
     <row r="87" spans="1:4" ht="124.2" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
@@ -8660,20 +9529,20 @@
       <c r="D97" s="6"/>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A98" s="28" t="s">
+      <c r="A98" s="31" t="s">
         <v>407</v>
       </c>
-      <c r="B98" s="29"/>
-      <c r="C98" s="29"/>
-      <c r="D98" s="30"/>
+      <c r="B98" s="32"/>
+      <c r="C98" s="32"/>
+      <c r="D98" s="33"/>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A99" s="25" t="s">
+      <c r="A99" s="28" t="s">
         <v>246</v>
       </c>
-      <c r="B99" s="26"/>
-      <c r="C99" s="26"/>
-      <c r="D99" s="27"/>
+      <c r="B99" s="29"/>
+      <c r="C99" s="29"/>
+      <c r="D99" s="30"/>
     </row>
     <row r="100" spans="1:4" ht="69" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
@@ -8810,12 +9679,12 @@
       <c r="D110" s="6"/>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A111" s="25" t="s">
+      <c r="A111" s="28" t="s">
         <v>266</v>
       </c>
-      <c r="B111" s="26"/>
-      <c r="C111" s="26"/>
-      <c r="D111" s="27"/>
+      <c r="B111" s="29"/>
+      <c r="C111" s="29"/>
+      <c r="D111" s="30"/>
     </row>
     <row r="112" spans="1:4" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A112" s="4" t="s">
@@ -8952,12 +9821,12 @@
       <c r="D122" s="6"/>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A123" s="25" t="s">
+      <c r="A123" s="28" t="s">
         <v>288</v>
       </c>
-      <c r="B123" s="26"/>
-      <c r="C123" s="26"/>
-      <c r="D123" s="27"/>
+      <c r="B123" s="29"/>
+      <c r="C123" s="29"/>
+      <c r="D123" s="30"/>
     </row>
     <row r="124" spans="1:4" ht="69" x14ac:dyDescent="0.3">
       <c r="A124" s="4" t="s">
@@ -9100,12 +9969,12 @@
       <c r="D135" s="6"/>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A136" s="25" t="s">
+      <c r="A136" s="28" t="s">
         <v>311</v>
       </c>
-      <c r="B136" s="26"/>
-      <c r="C136" s="26"/>
-      <c r="D136" s="27"/>
+      <c r="B136" s="29"/>
+      <c r="C136" s="29"/>
+      <c r="D136" s="30"/>
     </row>
     <row r="137" spans="1:4" ht="69" x14ac:dyDescent="0.3">
       <c r="A137" s="4" t="s">
@@ -9252,12 +10121,12 @@
       <c r="D148" s="6"/>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A149" s="25" t="s">
+      <c r="A149" s="28" t="s">
         <v>335</v>
       </c>
-      <c r="B149" s="26"/>
-      <c r="C149" s="26"/>
-      <c r="D149" s="27"/>
+      <c r="B149" s="29"/>
+      <c r="C149" s="29"/>
+      <c r="D149" s="30"/>
     </row>
     <row r="150" spans="1:4" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A150" s="4" t="s">
@@ -9394,12 +10263,12 @@
       <c r="D160" s="6"/>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A161" s="25" t="s">
+      <c r="A161" s="28" t="s">
         <v>356</v>
       </c>
-      <c r="B161" s="26"/>
-      <c r="C161" s="26"/>
-      <c r="D161" s="27"/>
+      <c r="B161" s="29"/>
+      <c r="C161" s="29"/>
+      <c r="D161" s="30"/>
     </row>
     <row r="162" spans="1:4" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A162" s="4" t="s">
@@ -9537,11 +10406,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A50:D50"/>
     <mergeCell ref="A62:D62"/>
     <mergeCell ref="A86:D86"/>
     <mergeCell ref="A98:D98"/>
@@ -9552,6 +10416,11 @@
     <mergeCell ref="A111:D111"/>
     <mergeCell ref="A99:D99"/>
     <mergeCell ref="A74:D74"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A50:D50"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -9581,11 +10450,11 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="34" t="s">
         <v>593</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
     </row>
     <row r="3" spans="1:3" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
@@ -9654,11 +10523,11 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="33" t="s">
+      <c r="A9" s="35" t="s">
         <v>594</v>
       </c>
-      <c r="B9" s="33"/>
-      <c r="C9" s="33"/>
+      <c r="B9" s="35"/>
+      <c r="C9" s="35"/>
     </row>
     <row r="10" spans="1:3" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
@@ -9727,11 +10596,11 @@
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="33" t="s">
+      <c r="A16" s="35" t="s">
         <v>595</v>
       </c>
-      <c r="B16" s="33"/>
-      <c r="C16" s="33"/>
+      <c r="B16" s="35"/>
+      <c r="C16" s="35"/>
     </row>
     <row r="17" spans="1:3" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
@@ -9800,11 +10669,11 @@
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="33" t="s">
+      <c r="A23" s="35" t="s">
         <v>596</v>
       </c>
-      <c r="B23" s="33"/>
-      <c r="C23" s="33"/>
+      <c r="B23" s="35"/>
+      <c r="C23" s="35"/>
     </row>
     <row r="24" spans="1:3" ht="96.6" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
@@ -9894,10 +10763,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="36" t="s">
         <v>659</v>
       </c>
-      <c r="B1" s="34"/>
+      <c r="B1" s="36"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
@@ -9956,10 +10825,10 @@
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="33" t="s">
+      <c r="A9" s="35" t="s">
         <v>658</v>
       </c>
-      <c r="B9" s="33"/>
+      <c r="B9" s="35"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">

</xml_diff>